<commit_message>
cases file rows added
</commit_message>
<xml_diff>
--- a/research/SA-2026-001-digital-evolution/data/Federal_Human_Trafficking_Prosecution_Explorer.xlsx
+++ b/research/SA-2026-001-digital-evolution/data/Federal_Human_Trafficking_Prosecution_Explorer.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="124">
   <si>
     <t>Case ID</t>
   </si>
@@ -91,6 +91,378 @@
   </si>
   <si>
     <t>Alleged use of a social media platform to recruit women, an online account for commercial-sex advertisements, edited digital photographs, and electronic funds transfers. Treat all conduct as allegations.</t>
+  </si>
+  <si>
+    <t>HT-2026-002</t>
+  </si>
+  <si>
+    <t>2026-07-16</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>Northern District of California</t>
+  </si>
+  <si>
+    <t>FBI; Oakland Police Department</t>
+  </si>
+  <si>
+    <t>Sex trafficking by force, fraud, or coercion</t>
+  </si>
+  <si>
+    <t>Commercial sex / online advertising / hotels</t>
+  </si>
+  <si>
+    <t>Michael Simon</t>
+  </si>
+  <si>
+    <t>Conspiracy to commit human trafficking by force, fraud, or coercion</t>
+  </si>
+  <si>
+    <t>Guilty plea; sentencing scheduled for 2026-10-01</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/usao-ndca/pr/oakland-man-pleads-guilty-conspiracy-commit-human-trafficking-oakland-blade</t>
+    </r>
+  </si>
+  <si>
+    <t>Defendant admitted participating in a trafficking conspiracy from June 2023 through September 2025. Victims were advertised online and housed in Oakland hotel rooms. Cellphones and text messages were used to communicate with prospective customers, direct victims to hotel rooms, and instruct victims to post online advertisements. The defendant admitted using physical violence when victims refused instructions or did not surrender proceeds.</t>
+  </si>
+  <si>
+    <t>HT-2026-003</t>
+  </si>
+  <si>
+    <t>2026-06-09</t>
+  </si>
+  <si>
+    <t>FL</t>
+  </si>
+  <si>
+    <t>Middle District of Florida</t>
+  </si>
+  <si>
+    <t>FBI; Homeland Security Investigations; Department of Labor</t>
+  </si>
+  <si>
+    <t>Forced labor</t>
+  </si>
+  <si>
+    <t>Agriculture / farm labor contracting</t>
+  </si>
+  <si>
+    <t>Alexander Villatoro Moreno</t>
+  </si>
+  <si>
+    <t>Conspiracy under the Racketeer Influenced and Corrupt Organizations Act</t>
+  </si>
+  <si>
+    <t>Sentenced to 70 months in prison; three years supervised release; restitution ordered</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/opa/pr/illegal-alien-sentenced-multi-state-racketeering-conspiracy-involving-forced-labor-mexican</t>
+    </r>
+  </si>
+  <si>
+    <t>The defendant pleaded guilty for his role in a multi-state forced-labor scheme involving H-2A agricultural workers. Court records described fraudulent recruitment, excessive recruitment fees, false promises about pay and working conditions, confiscated passports, debt, threats of arrest or deportation, isolation, poor living conditions, and threats against workers’ families. The enterprise operated in Florida, Kentucky, Indiana, Georgia, and North Carolina. This row uses Florida because the prosecution occurred in the Middle District of Florida.</t>
+  </si>
+  <si>
+    <t>HT-2026-004</t>
+  </si>
+  <si>
+    <t>2026-02-23</t>
+  </si>
+  <si>
+    <t>NC</t>
+  </si>
+  <si>
+    <t>Eastern District of North Carolina</t>
+  </si>
+  <si>
+    <t>Homeland Security Investigations; U.S. Department of Labor Office of Inspector General</t>
+  </si>
+  <si>
+    <t>Forced labor / labor trafficking</t>
+  </si>
+  <si>
+    <t>Agriculture / farm labor contracting / plant nurseries</t>
+  </si>
+  <si>
+    <t>Martha Zeferino Jose; Jose Rodriguez Munoz; Jeremy Zeferino Jose</t>
+  </si>
+  <si>
+    <t>Forced labor; conspiracy to commit forced labor; document servitude; alien harboring for financial gain; related visa fraud and obstruction charges</t>
+  </si>
+  <si>
+    <t>Indicted / charged; defendants presumed innocent</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/opa/pr/three-mexican-citizens-charged-trafficking-agricultural-workers-servitude-farms-virginia</t>
+    </r>
+  </si>
+  <si>
+    <t>The indictment alleges that workers were recruited from Mexico through the H-2A visa program using promises of lawful employment. Workers were allegedly charged recruitment fees, placed in debt, deprived of passports and identification documents, underpaid, housed in poor conditions, isolated, and threatened with arrest or deportation. Alleged labor occurred at farms and plant nurseries in North Carolina, Virginia, and Florida. Treat all conduct as allegations unless established through a plea or conviction.</t>
+  </si>
+  <si>
+    <t>HT-2026-005</t>
+  </si>
+  <si>
+    <t>2026-07-24</t>
+  </si>
+  <si>
+    <t>IL</t>
+  </si>
+  <si>
+    <t>Northern District of Illinois</t>
+  </si>
+  <si>
+    <t>Homeland Security Investigations; Lake County Sheriff’s Office</t>
+  </si>
+  <si>
+    <t>Multiple jobs / coerced wage labor</t>
+  </si>
+  <si>
+    <t>Gladys Ibanez-Olea</t>
+  </si>
+  <si>
+    <t>Bringing unauthorized individuals into the United States; obtaining forced labor through serious harm, abuse, and threats</t>
+  </si>
+  <si>
+    <t>Sentenced to 108 months in federal prison on 2026-07-21</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/usao-ndil/pr/cartel-member-who-trafficked-victims-mexico-chicagoland-forced-labor-sentenced-more-9</t>
+    </r>
+  </si>
+  <si>
+    <t>Defendant recruited victims in Mexico, arranged for them to be smuggled into the United States, housed them in Highland Park, Illinois, and forced them to work multiple jobs. She took their earnings as payment for alleged debts and used threats, harsh conditions, and threats against victims’ families to maintain control. Defendant pleaded guilty in February 2026 and was sentenced in July 2026.</t>
+  </si>
+  <si>
+    <t>HT-2026-006</t>
+  </si>
+  <si>
+    <t>2026-07-23</t>
+  </si>
+  <si>
+    <t>ME</t>
+  </si>
+  <si>
+    <t>District of Maine</t>
+  </si>
+  <si>
+    <t>Homeland Security Investigations New England</t>
+  </si>
+  <si>
+    <t>Commercial sex</t>
+  </si>
+  <si>
+    <t>Shawn Bonneau</t>
+  </si>
+  <si>
+    <t>Sex trafficking by force, fraud, or coercion; wire fraud</t>
+  </si>
+  <si>
+    <t>Indicted / charged; defendant presumed innocent</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/opa/pr/california-man-indicted-maine-sex-trafficking-and-related-offenses</t>
+    </r>
+  </si>
+  <si>
+    <t>The indictment alleges that from January 2016 through December 2023, the defendant compelled three adult women to perform commercial sex acts in Maine and elsewhere for his financial benefit. He is also alleged to have used electronic mail to fraudulently obtain money from another person while operating the trafficking scheme. Treat all conduct as allegations unless established through a plea or conviction.</t>
+  </si>
+  <si>
+    <t>HT-2026-007</t>
+  </si>
+  <si>
+    <t>2026-07-22</t>
+  </si>
+  <si>
+    <t>MO</t>
+  </si>
+  <si>
+    <t>Eastern District of Missouri</t>
+  </si>
+  <si>
+    <t>FBI Child Exploitation and Human Trafficking Task Force; St. Louis County Police Department</t>
+  </si>
+  <si>
+    <t>Sex trafficking of a minor</t>
+  </si>
+  <si>
+    <t>Social media / online advertising / hotel</t>
+  </si>
+  <si>
+    <t>Mack Mitchell</t>
+  </si>
+  <si>
+    <t>Guilty plea; sentencing scheduled for 2026-10-21</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/usao-edmo/pr/memphis-man-pleads-guilty-child-sex-trafficking-eve-trial</t>
+    </r>
+  </si>
+  <si>
+    <t>Defendant admitted meeting the victim through the Tag social media app when she was approximately 14 and corresponding with her for several years. In February 2024, he arranged an Uber to transport her from foster care, took her to a casino hotel, and had an associate photograph her and post advertisements online. The victim engaged in commercial sex acts and the proceeds were transferred to the defendant.</t>
+  </si>
+  <si>
+    <t>HT-2026-008</t>
+  </si>
+  <si>
+    <t>2026-07-28</t>
+  </si>
+  <si>
+    <t>TX</t>
+  </si>
+  <si>
+    <t>Northern District of Texas</t>
+  </si>
+  <si>
+    <t>Homeland Security Investigations; IRS Criminal Investigation; Dallas Police Department</t>
+  </si>
+  <si>
+    <t>Sex trafficking by force, fraud, or coercion; sex trafficking of a minor</t>
+  </si>
+  <si>
+    <t>Adult bookstore / commercial sex / arcade rooms</t>
+  </si>
+  <si>
+    <t>Aaron Tyrone Betford; Montre Lamont Mason; Eileen Mason; Trelynn Love Mason; Larry Jones; Krishenda Doss; Reginald Rose; Antonio Dario Osorio-Avelar</t>
+  </si>
+  <si>
+    <t>Conspiracy to commit sex trafficking; sex trafficking by force, fraud, or coercion; sex trafficking of a minor; conspiracy to launder monetary instruments; related firearm charges</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/usao-ndtx/pr/federal-state-and-local-law-enforcement-shut-down-dallas-sex-trafficking-conspiracy</t>
+    </r>
+  </si>
+  <si>
+    <t>The indictment alleges that eight defendants participated in a years-long sex-trafficking and money-laundering conspiracy operated through the Paris Adult Bookstore in Dallas. The business allegedly rented private arcade rooms for commercial sex acts and financially benefited from transactions involving women and minors. Six defendants were arrested, and 21 firearms were recovered. Treat all conduct as allegations unless established through a plea or conviction.</t>
+  </si>
+  <si>
+    <t>HT-2026-009</t>
+  </si>
+  <si>
+    <t>NE</t>
+  </si>
+  <si>
+    <t>District of Nebraska</t>
+  </si>
+  <si>
+    <t>Omaha Police Department–Homeland Security Investigations Human Trafficking Task Force</t>
+  </si>
+  <si>
+    <t>Sex trafficking of minors by force, fraud, or coercion</t>
+  </si>
+  <si>
+    <t>Online commercial sex / hotel</t>
+  </si>
+  <si>
+    <t>Eduardo Jose Perdomo</t>
+  </si>
+  <si>
+    <t>Sex trafficking of two minors by force, fraud, or coercion</t>
+  </si>
+  <si>
+    <t>Sentenced to 240 months in prison; five years of supervised release; $5,400 restitution</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/usao-ne/pr/venezuelan-man-sentenced-sex-trafficking-minors</t>
+    </r>
+  </si>
+  <si>
+    <t>Defendant transported two minor victims, ages 15 and 16, from another state to an Omaha hotel. He coordinated with a co-defendant to advertise the victims online and communicate with prospective buyers. He also arranged for hotel staff to receive commercial sex acts in exchange for allowing the operation to continue at the hotel. The trafficking was identified after officers responded to an unrelated theft report and recognized indicators of exploitation.</t>
+  </si>
+  <si>
+    <t>HT-2026-010</t>
+  </si>
+  <si>
+    <t>Eastern District of New York</t>
+  </si>
+  <si>
+    <t>FBI New York Field Office; FBI Newark Field Office</t>
+  </si>
+  <si>
+    <t>Sex trafficking of minors; sex trafficking by force, fraud, or coercion</t>
+  </si>
+  <si>
+    <t>Hotels / online advertising / commercial sex</t>
+  </si>
+  <si>
+    <t>Tyrone Stylistic Crooks</t>
+  </si>
+  <si>
+    <t>Sex trafficking; sexual exploitation of minors; transportation for prostitution</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://www.justice.gov/usao-edny/pr/queens-man-indicted-sex-trafficking-five-victims-including-three-minors-hotels-long</t>
+    </r>
+  </si>
+  <si>
+    <t>The indictment alleges that the defendant trafficked five victims, including three minors, at hotels in New York and elsewhere. He allegedly used text messages and other online communications to recruit victims, paid for travel, created and posted online advertisements, arranged commercial sex transactions, controlled proceeds, and used fraud, threats, and violence. Treat all conduct as allegations unless established through a plea or conviction.</t>
   </si>
 </sst>
 </file>
@@ -154,7 +526,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="13"/>
+        <fgColor indexed="12"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -165,7 +537,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -190,7 +562,7 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="12"/>
+        <color indexed="13"/>
       </left>
       <right/>
       <top style="thin">
@@ -245,7 +617,7 @@
         <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="12"/>
+        <color indexed="13"/>
       </right>
       <top style="thin">
         <color indexed="11"/>
@@ -297,6 +669,68 @@
       </top>
       <bottom style="thin">
         <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="13"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="13"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="13"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="13"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="13"/>
       </bottom>
       <diagonal/>
     </border>
@@ -306,7 +740,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -319,28 +753,46 @@
     <xf numFmtId="49" fontId="4" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -363,8 +815,8 @@
       <rgbColor rgb="ffbdc0bf"/>
       <rgbColor rgb="ffa5a5a5"/>
       <rgbColor rgb="ff3f3f3f"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
-      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ff0000ff"/>
       <rgbColor rgb="ffdbdbdb"/>
     </indexedColors>
@@ -1428,7 +1880,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="12" width="16.3516" style="1" customWidth="1"/>
@@ -1512,106 +1964,387 @@
       </c>
     </row>
     <row r="3" ht="20.05" customHeight="1">
-      <c r="A3" s="9"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="11"/>
-      <c r="E3" s="11"/>
-      <c r="F3" s="11"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
+      <c r="A3" t="s" s="9">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s" s="10">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s" s="11">
+        <v>26</v>
+      </c>
+      <c r="D3" t="s" s="11">
+        <v>27</v>
+      </c>
+      <c r="E3" t="s" s="11">
+        <v>28</v>
+      </c>
+      <c r="F3" t="s" s="11">
+        <v>29</v>
+      </c>
+      <c r="G3" t="s" s="11">
+        <v>30</v>
+      </c>
+      <c r="H3" t="s" s="11">
+        <v>31</v>
+      </c>
+      <c r="I3" t="s" s="11">
+        <v>32</v>
+      </c>
+      <c r="J3" t="s" s="11">
+        <v>33</v>
+      </c>
+      <c r="K3" t="s" s="11">
+        <v>34</v>
+      </c>
+      <c r="L3" t="s" s="11">
+        <v>35</v>
+      </c>
     </row>
     <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" s="9"/>
-      <c r="B4" s="10"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
+      <c r="A4" t="s" s="9">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s" s="10">
+        <v>37</v>
+      </c>
+      <c r="C4" t="s" s="11">
+        <v>38</v>
+      </c>
+      <c r="D4" t="s" s="11">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s" s="11">
+        <v>40</v>
+      </c>
+      <c r="F4" t="s" s="11">
+        <v>41</v>
+      </c>
+      <c r="G4" t="s" s="11">
+        <v>42</v>
+      </c>
+      <c r="H4" t="s" s="11">
+        <v>43</v>
+      </c>
+      <c r="I4" t="s" s="11">
+        <v>44</v>
+      </c>
+      <c r="J4" t="s" s="11">
+        <v>45</v>
+      </c>
+      <c r="K4" t="s" s="11">
+        <v>46</v>
+      </c>
+      <c r="L4" t="s" s="11">
+        <v>47</v>
+      </c>
     </row>
     <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" s="9"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
+      <c r="A5" t="s" s="9">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s" s="10">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s" s="11">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s" s="11">
+        <v>51</v>
+      </c>
+      <c r="E5" t="s" s="11">
+        <v>52</v>
+      </c>
+      <c r="F5" t="s" s="11">
+        <v>53</v>
+      </c>
+      <c r="G5" t="s" s="11">
+        <v>54</v>
+      </c>
+      <c r="H5" t="s" s="11">
+        <v>55</v>
+      </c>
+      <c r="I5" t="s" s="11">
+        <v>56</v>
+      </c>
+      <c r="J5" t="s" s="11">
+        <v>57</v>
+      </c>
+      <c r="K5" t="s" s="11">
+        <v>58</v>
+      </c>
+      <c r="L5" t="s" s="11">
+        <v>59</v>
+      </c>
     </row>
     <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" s="9"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
+      <c r="A6" t="s" s="9">
+        <v>60</v>
+      </c>
+      <c r="B6" t="s" s="10">
+        <v>61</v>
+      </c>
+      <c r="C6" t="s" s="11">
+        <v>62</v>
+      </c>
+      <c r="D6" t="s" s="11">
+        <v>63</v>
+      </c>
+      <c r="E6" t="s" s="11">
+        <v>64</v>
+      </c>
+      <c r="F6" t="s" s="11">
+        <v>53</v>
+      </c>
+      <c r="G6" t="s" s="11">
+        <v>65</v>
+      </c>
+      <c r="H6" t="s" s="11">
+        <v>66</v>
+      </c>
+      <c r="I6" t="s" s="11">
+        <v>67</v>
+      </c>
+      <c r="J6" t="s" s="11">
+        <v>68</v>
+      </c>
+      <c r="K6" t="s" s="11">
+        <v>69</v>
+      </c>
+      <c r="L6" t="s" s="11">
+        <v>70</v>
+      </c>
     </row>
     <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" s="9"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
+      <c r="A7" t="s" s="9">
+        <v>71</v>
+      </c>
+      <c r="B7" t="s" s="10">
+        <v>72</v>
+      </c>
+      <c r="C7" t="s" s="11">
+        <v>73</v>
+      </c>
+      <c r="D7" t="s" s="11">
+        <v>74</v>
+      </c>
+      <c r="E7" t="s" s="11">
+        <v>75</v>
+      </c>
+      <c r="F7" t="s" s="11">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s" s="11">
+        <v>76</v>
+      </c>
+      <c r="H7" t="s" s="11">
+        <v>77</v>
+      </c>
+      <c r="I7" t="s" s="11">
+        <v>78</v>
+      </c>
+      <c r="J7" t="s" s="11">
+        <v>79</v>
+      </c>
+      <c r="K7" t="s" s="11">
+        <v>80</v>
+      </c>
+      <c r="L7" t="s" s="11">
+        <v>81</v>
+      </c>
     </row>
     <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" s="9"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
+      <c r="A8" t="s" s="9">
+        <v>82</v>
+      </c>
+      <c r="B8" t="s" s="10">
+        <v>83</v>
+      </c>
+      <c r="C8" t="s" s="11">
+        <v>84</v>
+      </c>
+      <c r="D8" t="s" s="11">
+        <v>85</v>
+      </c>
+      <c r="E8" t="s" s="11">
+        <v>86</v>
+      </c>
+      <c r="F8" t="s" s="11">
+        <v>87</v>
+      </c>
+      <c r="G8" t="s" s="11">
+        <v>88</v>
+      </c>
+      <c r="H8" t="s" s="11">
+        <v>89</v>
+      </c>
+      <c r="I8" t="s" s="11">
+        <v>87</v>
+      </c>
+      <c r="J8" t="s" s="11">
+        <v>90</v>
+      </c>
+      <c r="K8" t="s" s="11">
+        <v>91</v>
+      </c>
+      <c r="L8" t="s" s="11">
+        <v>92</v>
+      </c>
     </row>
     <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
+      <c r="A9" t="s" s="9">
+        <v>93</v>
+      </c>
+      <c r="B9" t="s" s="10">
+        <v>94</v>
+      </c>
+      <c r="C9" t="s" s="11">
+        <v>95</v>
+      </c>
+      <c r="D9" t="s" s="11">
+        <v>96</v>
+      </c>
+      <c r="E9" t="s" s="11">
+        <v>97</v>
+      </c>
+      <c r="F9" t="s" s="11">
+        <v>98</v>
+      </c>
+      <c r="G9" t="s" s="11">
+        <v>99</v>
+      </c>
+      <c r="H9" t="s" s="11">
+        <v>100</v>
+      </c>
+      <c r="I9" t="s" s="11">
+        <v>101</v>
+      </c>
+      <c r="J9" t="s" s="11">
+        <v>57</v>
+      </c>
+      <c r="K9" t="s" s="11">
+        <v>102</v>
+      </c>
+      <c r="L9" t="s" s="11">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" ht="20.05" customHeight="1">
+      <c r="A10" t="s" s="9">
+        <v>104</v>
+      </c>
+      <c r="B10" t="s" s="10">
+        <v>83</v>
+      </c>
+      <c r="C10" t="s" s="11">
+        <v>105</v>
+      </c>
+      <c r="D10" t="s" s="11">
+        <v>106</v>
+      </c>
+      <c r="E10" t="s" s="11">
+        <v>107</v>
+      </c>
+      <c r="F10" t="s" s="11">
+        <v>108</v>
+      </c>
+      <c r="G10" t="s" s="11">
+        <v>109</v>
+      </c>
+      <c r="H10" t="s" s="11">
+        <v>110</v>
+      </c>
+      <c r="I10" t="s" s="11">
+        <v>111</v>
+      </c>
+      <c r="J10" t="s" s="11">
+        <v>112</v>
+      </c>
+      <c r="K10" t="s" s="11">
+        <v>113</v>
+      </c>
+      <c r="L10" t="s" s="11">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="11" ht="20.05" customHeight="1">
+      <c r="A11" t="s" s="9">
+        <v>115</v>
+      </c>
+      <c r="B11" t="s" s="10">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s" s="11">
+        <v>14</v>
+      </c>
+      <c r="D11" t="s" s="11">
+        <v>116</v>
+      </c>
+      <c r="E11" t="s" s="11">
+        <v>117</v>
+      </c>
+      <c r="F11" t="s" s="11">
+        <v>118</v>
+      </c>
+      <c r="G11" t="s" s="11">
+        <v>119</v>
+      </c>
+      <c r="H11" t="s" s="11">
+        <v>120</v>
+      </c>
+      <c r="I11" t="s" s="11">
+        <v>121</v>
+      </c>
+      <c r="J11" t="s" s="11">
+        <v>79</v>
+      </c>
+      <c r="K11" t="s" s="11">
+        <v>122</v>
+      </c>
+      <c r="L11" t="s" s="11">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="12" ht="14.7" customHeight="1">
+      <c r="A12" s="12"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="14"/>
+    </row>
+    <row r="13" ht="14.7" customHeight="1">
+      <c r="A13" s="15"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="16"/>
+      <c r="I13" s="16"/>
+      <c r="J13" s="16"/>
+      <c r="K13" s="16"/>
+      <c r="L13" s="17"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="K2" r:id="rId1" location="" tooltip="" display="https://www.justice.gov/usao-sdny/pr/us-attorneys-office-and-fbi-continue-their-fight-against-sex-trafficking-new-york"/>
+    <hyperlink ref="K3" r:id="rId2" location="" tooltip="" display="https://www.justice.gov/usao-ndca/pr/oakland-man-pleads-guilty-conspiracy-commit-human-trafficking-oakland-blade"/>
+    <hyperlink ref="K4" r:id="rId3" location="" tooltip="" display="https://www.justice.gov/opa/pr/illegal-alien-sentenced-multi-state-racketeering-conspiracy-involving-forced-labor-mexican"/>
+    <hyperlink ref="K5" r:id="rId4" location="" tooltip="" display="https://www.justice.gov/opa/pr/three-mexican-citizens-charged-trafficking-agricultural-workers-servitude-farms-virginia"/>
+    <hyperlink ref="K6" r:id="rId5" location="" tooltip="" display="https://www.justice.gov/usao-ndil/pr/cartel-member-who-trafficked-victims-mexico-chicagoland-forced-labor-sentenced-more-9"/>
+    <hyperlink ref="K7" r:id="rId6" location="" tooltip="" display="https://www.justice.gov/opa/pr/california-man-indicted-maine-sex-trafficking-and-related-offenses"/>
+    <hyperlink ref="K8" r:id="rId7" location="" tooltip="" display="https://www.justice.gov/usao-edmo/pr/memphis-man-pleads-guilty-child-sex-trafficking-eve-trial"/>
+    <hyperlink ref="K9" r:id="rId8" location="" tooltip="" display="https://www.justice.gov/usao-ndtx/pr/federal-state-and-local-law-enforcement-shut-down-dallas-sex-trafficking-conspiracy"/>
+    <hyperlink ref="K10" r:id="rId9" location="" tooltip="" display="https://www.justice.gov/usao-ne/pr/venezuelan-man-sentenced-sex-trafficking-minors"/>
+    <hyperlink ref="K11" r:id="rId10" location="" tooltip="" display="https://www.justice.gov/usao-edny/pr/queens-man-indicted-sex-trafficking-five-victims-including-three-minors-hotels-long"/>
   </hyperlinks>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>